<commit_message>
Implement E2E test workflow and push project updates
</commit_message>
<xml_diff>
--- a/E2E_Test_Report_V2.xlsx
+++ b/E2E_Test_Report_V2.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G29"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -447,13 +447,13 @@
         <v>Eco-Pantry title, Sign In/Create Account tabs visible</v>
       </c>
       <c r="E2" t="str">
-        <v>Eco-Pantry branding ✓, Sign In tab ✓, Create Account tab ✓</v>
+        <v>Eco-Pantry branding ✗, Sign In tab ✗, Create Account tab ✗</v>
       </c>
       <c r="F2" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G2" t="str">
-        <v>13/6/2026, 10:34:18 am</v>
+        <v>18/6/2026, 1:42:24 pm</v>
       </c>
     </row>
     <row r="3">
@@ -470,662 +470,616 @@
         <v>Dashboard loads, Welcome greeting shown</v>
       </c>
       <c r="E3" t="str">
-        <v>Successfully authenticated and dashboard rendered with pantry data</v>
+        <v>Login processed, app state transitioned</v>
       </c>
       <c r="F3" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G3" t="str">
-        <v>13/6/2026, 10:34:24 am</v>
+        <v>18/6/2026, 1:42:36 pm</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>TC-03</v>
+        <v>TC-04</v>
       </c>
       <c r="B4" t="str">
         <v>Authentication</v>
       </c>
       <c r="C4" t="str">
-        <v>Login with invalid password</v>
+        <v>Login with empty fields</v>
       </c>
       <c r="D4" t="str">
-        <v>Error message displayed</v>
+        <v>Validation error "Please fill in all credentials"</v>
       </c>
       <c r="E4" t="str">
-        <v>Invalid credentials rejected, user remains on login page with error feedback</v>
+        <v>No validation</v>
       </c>
       <c r="F4" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G4" t="str">
-        <v>13/6/2026, 10:34:29 am</v>
+        <v>18/6/2026, 1:43:13 pm</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>TC-04</v>
+        <v>TC-06</v>
       </c>
       <c r="B5" t="str">
         <v>Authentication</v>
       </c>
       <c r="C5" t="str">
-        <v>Login with empty fields</v>
+        <v>Logout functionality</v>
       </c>
       <c r="D5" t="str">
-        <v>Validation error "Please fill in all credentials"</v>
+        <v>Returns to login page</v>
       </c>
       <c r="E5" t="str">
-        <v>Empty submission blocked, validation error shown to user</v>
+        <v>Logout executed</v>
       </c>
       <c r="F5" t="str">
         <v>PASS</v>
       </c>
       <c r="G5" t="str">
-        <v>13/6/2026, 10:34:33 am</v>
+        <v>18/6/2026, 1:43:48 pm</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>TC-05</v>
+        <v>TC-07</v>
       </c>
       <c r="B6" t="str">
-        <v>Authentication</v>
+        <v>Dashboard</v>
       </c>
       <c r="C6" t="str">
-        <v>Switch between Sign In and Create Account tabs</v>
+        <v>Dashboard loads after login</v>
       </c>
       <c r="D6" t="str">
-        <v>Tab UI toggles, correct fields shown</v>
+        <v>Header "Eco-Pantry", user greeting visible</v>
       </c>
       <c r="E6" t="str">
-        <v>Create Account shows Display Name ✓ and Family Code ✓. Switching back hides signup fields</v>
+        <v>Dashboard header "Eco-Pantry" ✗, Welcome greeting</v>
       </c>
       <c r="F6" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G6" t="str">
-        <v>13/6/2026, 10:34:37 am</v>
+        <v>18/6/2026, 1:43:51 pm</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>TC-06</v>
+        <v>TC-08</v>
       </c>
       <c r="B7" t="str">
-        <v>Authentication</v>
+        <v>Dashboard</v>
       </c>
       <c r="C7" t="str">
-        <v>Logout functionality</v>
+        <v>Expiring Soon section visible</v>
       </c>
       <c r="D7" t="str">
-        <v>Returns to login page</v>
+        <v>Section title with Clock icon present</v>
       </c>
       <c r="E7" t="str">
-        <v>Logout successful, user session cleared, redirected to Sign In page</v>
+        <v>Section not found in active slide</v>
       </c>
       <c r="F7" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G7" t="str">
-        <v>13/6/2026, 10:34:45 am</v>
+        <v>18/6/2026, 1:43:51 pm</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>TC-07</v>
+        <v>TC-09</v>
       </c>
       <c r="B8" t="str">
         <v>Dashboard</v>
       </c>
       <c r="C8" t="str">
-        <v>Dashboard loads after login</v>
+        <v>My Eco-Pantry section visible</v>
       </c>
       <c r="D8" t="str">
-        <v>Header "Eco-Pantry", user greeting visible</v>
+        <v>Section title and search input present</v>
       </c>
       <c r="E8" t="str">
-        <v>Dashboard header "Eco-Pantry" ✓, Welcome greeting ✓</v>
+        <v>Section not found</v>
       </c>
       <c r="F8" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G8" t="str">
-        <v>13/6/2026, 10:34:54 am</v>
+        <v>18/6/2026, 1:43:51 pm</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>TC-08</v>
+        <v>TC-10</v>
       </c>
       <c r="B9" t="str">
         <v>Dashboard</v>
       </c>
       <c r="C9" t="str">
-        <v>Expiring Soon section visible</v>
+        <v>Smart Grocery Anti-List visible</v>
       </c>
       <c r="D9" t="str">
-        <v>Section title with Clock icon present</v>
+        <v>Section title present with item chips</v>
       </c>
       <c r="E9" t="str">
-        <v>"Expiring Soon" section rendered with Clock icon and food item cards</v>
+        <v>Section not found</v>
       </c>
       <c r="F9" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G9" t="str">
-        <v>13/6/2026, 10:34:54 am</v>
+        <v>18/6/2026, 1:43:51 pm</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>TC-09</v>
+        <v>TC-11</v>
       </c>
       <c r="B10" t="str">
         <v>Dashboard</v>
       </c>
       <c r="C10" t="str">
-        <v>My Eco-Pantry section visible</v>
+        <v>Pantry search filter works</v>
       </c>
       <c r="D10" t="str">
-        <v>Section title and search input present</v>
+        <v>Items filter when typing</v>
       </c>
       <c r="E10" t="str">
-        <v>"My Eco-Pantry" inventory section rendered with search input</v>
+        <v>Search input not found</v>
       </c>
       <c r="F10" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G10" t="str">
-        <v>13/6/2026, 10:34:54 am</v>
+        <v>18/6/2026, 1:43:52 pm</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>TC-10</v>
+        <v>TC-12</v>
       </c>
       <c r="B11" t="str">
         <v>Dashboard</v>
       </c>
       <c r="C11" t="str">
-        <v>Smart Grocery Anti-List visible</v>
+        <v>"Scan New Items" button navigates to scanner</v>
       </c>
       <c r="D11" t="str">
-        <v>Section title present with item chips</v>
+        <v>Hash changes to #scanner</v>
       </c>
       <c r="E11" t="str">
-        <v>Smart Grocery Anti-List section displayed with in-stock/needed item chips</v>
+        <v>Scan button not found</v>
       </c>
       <c r="F11" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G11" t="str">
-        <v>13/6/2026, 10:34:54 am</v>
+        <v>18/6/2026, 1:43:53 pm</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>TC-11</v>
+        <v>TC-13</v>
       </c>
       <c r="B12" t="str">
-        <v>Dashboard</v>
+        <v>Navigation</v>
       </c>
       <c r="C12" t="str">
-        <v>Pantry search filter works</v>
+        <v>Navigate to Inventory Scanner</v>
       </c>
       <c r="D12" t="str">
-        <v>Items filter when typing</v>
+        <v>#scanner page loads</v>
       </c>
       <c r="E12" t="str">
-        <v>Search input accepts query and filters pantry inventory items in real-time</v>
+        <v>Hash: #scanner ✓. Page content keywords missing</v>
       </c>
       <c r="F12" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G12" t="str">
-        <v>13/6/2026, 10:34:56 am</v>
+        <v>18/6/2026, 1:43:56 pm</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>TC-12</v>
+        <v>TC-14</v>
       </c>
       <c r="B13" t="str">
-        <v>Dashboard</v>
+        <v>Navigation</v>
       </c>
       <c r="C13" t="str">
-        <v>"Scan New Items" button navigates to scanner</v>
+        <v>Navigate to Smart Recipes</v>
       </c>
       <c r="D13" t="str">
-        <v>Hash changes to #scanner</v>
+        <v>#recipes page loads</v>
       </c>
       <c r="E13" t="str">
-        <v>Button clicked, navigated to #scanner</v>
+        <v>Hash: #recipes ✓. Page content keywords missing</v>
       </c>
       <c r="F13" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G13" t="str">
-        <v>13/6/2026, 10:34:57 am</v>
+        <v>18/6/2026, 1:43:58 pm</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>TC-13</v>
+        <v>TC-15</v>
       </c>
       <c r="B14" t="str">
         <v>Navigation</v>
       </c>
       <c r="C14" t="str">
-        <v>Navigate to Inventory Scanner</v>
+        <v>Navigate to Sustainability Analytics</v>
       </c>
       <c r="D14" t="str">
-        <v>#scanner page loads</v>
+        <v>#analytics page loads</v>
       </c>
       <c r="E14" t="str">
-        <v>Hash: #scanner ✓. Page content keywords confirmed</v>
+        <v>Hash: #analytics ✓. Page content keywords missing</v>
       </c>
       <c r="F14" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G14" t="str">
-        <v>13/6/2026, 10:35:01 am</v>
+        <v>18/6/2026, 1:44:00 pm</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>TC-14</v>
+        <v>TC-16</v>
       </c>
       <c r="B15" t="str">
         <v>Navigation</v>
       </c>
       <c r="C15" t="str">
-        <v>Navigate to Smart Recipes</v>
+        <v>Navigate to Profile &amp; AI Settings</v>
       </c>
       <c r="D15" t="str">
-        <v>#recipes page loads</v>
+        <v>#profile page loads</v>
       </c>
       <c r="E15" t="str">
-        <v>Hash: #recipes ✓. Page content keywords confirmed</v>
+        <v>Hash: #profile ✓. Page content keywords missing</v>
       </c>
       <c r="F15" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G15" t="str">
-        <v>13/6/2026, 10:35:03 am</v>
+        <v>18/6/2026, 1:44:01 pm</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>TC-15</v>
+        <v>TC-17</v>
       </c>
       <c r="B16" t="str">
         <v>Navigation</v>
       </c>
       <c r="C16" t="str">
-        <v>Navigate to Sustainability Analytics</v>
+        <v>Navigate to Eco Community</v>
       </c>
       <c r="D16" t="str">
-        <v>#analytics page loads</v>
+        <v>#community page loads</v>
       </c>
       <c r="E16" t="str">
-        <v>Hash: #analytics ✓. Page content keywords confirmed</v>
+        <v>Hash: #community ✓. Page content keywords missing</v>
       </c>
       <c r="F16" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G16" t="str">
-        <v>13/6/2026, 10:35:04 am</v>
+        <v>18/6/2026, 1:44:03 pm</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>TC-16</v>
+        <v>TC-18</v>
       </c>
       <c r="B17" t="str">
         <v>Navigation</v>
       </c>
       <c r="C17" t="str">
-        <v>Navigate to Profile &amp; AI Settings</v>
+        <v>Navigate to Dashboard</v>
       </c>
       <c r="D17" t="str">
-        <v>#profile page loads</v>
+        <v>#dashboard page loads</v>
       </c>
       <c r="E17" t="str">
-        <v>Hash: #profile ✓. Page content keywords confirmed</v>
+        <v>Hash: #dashboard ✓. Page content keywords missing</v>
       </c>
       <c r="F17" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G17" t="str">
-        <v>13/6/2026, 10:35:06 am</v>
+        <v>18/6/2026, 1:44:04 pm</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>TC-17</v>
+        <v>TC-19</v>
       </c>
       <c r="B18" t="str">
-        <v>Navigation</v>
+        <v>Profile</v>
       </c>
       <c r="C18" t="str">
-        <v>Navigate to Eco Community</v>
+        <v>Profile page shows user info</v>
       </c>
       <c r="D18" t="str">
-        <v>#community page loads</v>
+        <v>Name, email, badge visible</v>
       </c>
       <c r="E18" t="str">
-        <v>Hash: #community ✓. Page content keywords confirmed</v>
+        <v>Profile section, Email, Badge/Tier</v>
       </c>
       <c r="F18" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G18" t="str">
-        <v>13/6/2026, 10:35:08 am</v>
+        <v>18/6/2026, 1:44:08 pm</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>TC-18</v>
+        <v>TC-20</v>
       </c>
       <c r="B19" t="str">
-        <v>Navigation</v>
+        <v>Profile</v>
       </c>
       <c r="C19" t="str">
-        <v>Navigate to Dashboard</v>
+        <v>Eco Points progress bar visible</v>
       </c>
       <c r="D19" t="str">
-        <v>#dashboard page loads</v>
+        <v>Points count and progress bar rendered</v>
       </c>
       <c r="E19" t="str">
-        <v>Hash: #dashboard ✓. Page content keywords confirmed</v>
+        <v>Eco Points, Progress bar</v>
       </c>
       <c r="F19" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G19" t="str">
-        <v>13/6/2026, 10:35:09 am</v>
+        <v>18/6/2026, 1:44:13 pm</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>TC-19</v>
+        <v>TC-21</v>
       </c>
       <c r="B20" t="str">
         <v>Profile</v>
       </c>
       <c r="C20" t="str">
-        <v>Profile page shows user info</v>
+        <v>Dietary restriction dropdown works</v>
       </c>
       <c r="D20" t="str">
-        <v>Name, email, badge visible</v>
+        <v>Dropdown changes value</v>
       </c>
       <c r="E20" t="str">
-        <v>Profile section ✓, Email ✓, Badge/Tier ✓</v>
+        <v>Select element not found</v>
       </c>
       <c r="F20" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G20" t="str">
-        <v>13/6/2026, 10:35:13 am</v>
+        <v>18/6/2026, 1:44:14 pm</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>TC-20</v>
+        <v>TC-22</v>
       </c>
       <c r="B21" t="str">
         <v>Profile</v>
       </c>
       <c r="C21" t="str">
-        <v>Eco Points progress bar visible</v>
+        <v>Household size selector works</v>
       </c>
       <c r="D21" t="str">
-        <v>Points count and progress bar rendered</v>
+        <v>Buttons toggle correctly</v>
       </c>
       <c r="E21" t="str">
-        <v>Eco Points ✓, Progress bar ✓</v>
+        <v>Household section present</v>
       </c>
       <c r="F21" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G21" t="str">
-        <v>13/6/2026, 10:35:13 am</v>
+        <v>18/6/2026, 1:44:14 pm</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>TC-21</v>
+        <v>TC-23</v>
       </c>
       <c r="B22" t="str">
-        <v>Profile</v>
+        <v>Recipes</v>
       </c>
       <c r="C22" t="str">
-        <v>Dietary restriction dropdown works</v>
+        <v>Recipes page loads</v>
       </c>
       <c r="D22" t="str">
-        <v>Dropdown changes value</v>
+        <v>"AI-Optimized" header visible</v>
       </c>
       <c r="E22" t="str">
-        <v>Dropdown toggled to "Vegan" successfully, then reset to None</v>
+        <v>Header keywords not found</v>
       </c>
       <c r="F22" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G22" t="str">
-        <v>13/6/2026, 10:35:14 am</v>
+        <v>18/6/2026, 1:44:18 pm</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>TC-22</v>
+        <v>TC-24</v>
       </c>
       <c r="B23" t="str">
-        <v>Profile</v>
+        <v>Recipes</v>
       </c>
       <c r="C23" t="str">
-        <v>Household size selector works</v>
+        <v>Generate with AI card visible</v>
       </c>
       <c r="D23" t="str">
-        <v>Buttons toggle correctly</v>
+        <v>Card with Sparkles icon present</v>
       </c>
       <c r="E23" t="str">
-        <v>Household Size section found, button "1" clicked</v>
+        <v>Generate card not found</v>
       </c>
       <c r="F23" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G23" t="str">
-        <v>13/6/2026, 10:35:15 am</v>
+        <v>18/6/2026, 1:44:18 pm</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>TC-23</v>
+        <v>TC-25</v>
       </c>
       <c r="B24" t="str">
         <v>Recipes</v>
       </c>
       <c r="C24" t="str">
-        <v>Recipes page loads</v>
+        <v>Recipe cards display if available</v>
       </c>
       <c r="D24" t="str">
-        <v>"AI-Optimized" header visible</v>
+        <v>Recipe cards with matchScore badge</v>
       </c>
       <c r="E24" t="str">
-        <v>AI-Optimized Zero-Waste Recipes header displayed on recipes page</v>
+        <v>0 recipe cards found. Recipe area rendered</v>
       </c>
       <c r="F24" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G24" t="str">
-        <v>13/6/2026, 10:35:19 am</v>
+        <v>18/6/2026, 1:44:18 pm</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>TC-24</v>
+        <v>TC-26</v>
       </c>
       <c r="B25" t="str">
-        <v>Recipes</v>
+        <v>Analytics</v>
       </c>
       <c r="C25" t="str">
-        <v>Generate with AI card visible</v>
+        <v>Analytics page loads</v>
       </c>
       <c r="D25" t="str">
-        <v>Card with Sparkles icon present</v>
+        <v>"Sustainability Analytics" header visible</v>
       </c>
       <c r="E25" t="str">
-        <v>"Generate with AI" card rendered with Sparkles icon for recipe generation</v>
+        <v>Analytics header not found</v>
       </c>
       <c r="F25" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G25" t="str">
-        <v>13/6/2026, 10:35:19 am</v>
+        <v>18/6/2026, 1:44:21 pm</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>TC-25</v>
+        <v>TC-27</v>
       </c>
       <c r="B26" t="str">
-        <v>Recipes</v>
+        <v>Analytics</v>
       </c>
       <c r="C26" t="str">
-        <v>Recipe cards display if available</v>
+        <v>Emergency Food Donation section visible</v>
       </c>
       <c r="D26" t="str">
-        <v>Recipe cards with matchScore badge</v>
+        <v>Donation section + "New Donation Request" button</v>
       </c>
       <c r="E26" t="str">
-        <v>1 recipe cards found. Recipe content confirmed</v>
+        <v>Section not found</v>
       </c>
       <c r="F26" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G26" t="str">
-        <v>13/6/2026, 10:35:19 am</v>
+        <v>18/6/2026, 1:44:21 pm</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>TC-26</v>
+        <v>TC-28</v>
       </c>
       <c r="B27" t="str">
         <v>Analytics</v>
       </c>
       <c r="C27" t="str">
-        <v>Analytics page loads</v>
+        <v>Donation modal opens</v>
       </c>
       <c r="D27" t="str">
-        <v>"Sustainability Analytics" header visible</v>
+        <v>Modal appears on button click</v>
       </c>
       <c r="E27" t="str">
-        <v>Sustainability Analytics page loaded with waste prediction charts and smart alerts</v>
+        <v>Donation Request button not found</v>
       </c>
       <c r="F27" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G27" t="str">
-        <v>13/6/2026, 10:35:23 am</v>
+        <v>18/6/2026, 1:44:23 pm</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>TC-27</v>
+        <v>TC-29</v>
       </c>
       <c r="B28" t="str">
-        <v>Analytics</v>
+        <v>AI Chatbot</v>
       </c>
       <c r="C28" t="str">
-        <v>Emergency Food Donation section visible</v>
+        <v>Chatbot bubble visible</v>
       </c>
       <c r="D28" t="str">
-        <v>Donation section + "New Donation Request" button</v>
+        <v>Floating chat bubble rendered</v>
       </c>
       <c r="E28" t="str">
-        <v>Donation section displayed with "New Donation Request" button</v>
+        <v>DOM exists: false, Visible: false</v>
       </c>
       <c r="F28" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G28" t="str">
-        <v>13/6/2026, 10:35:23 am</v>
+        <v>18/6/2026, 1:44:31 pm</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>TC-28</v>
+        <v>TC-30</v>
       </c>
       <c r="B29" t="str">
-        <v>Analytics</v>
+        <v>AI Chatbot</v>
       </c>
       <c r="C29" t="str">
-        <v>Donation modal opens</v>
+        <v>Chatbot opens and shows welcome message</v>
       </c>
       <c r="D29" t="str">
-        <v>Modal appears on button click</v>
+        <v>Chat pane opens</v>
       </c>
       <c r="E29" t="str">
-        <v>Donation modal opened with item selection list and NGO destination picker</v>
+        <v>Chatbot bubble not clickable</v>
       </c>
       <c r="F29" t="str">
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G29" t="str">
-        <v>13/6/2026, 10:35:25 am</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="str">
-        <v>TC-29</v>
-      </c>
-      <c r="B30" t="str">
-        <v>AI Chatbot</v>
-      </c>
-      <c r="C30" t="str">
-        <v>Chatbot bubble visible</v>
-      </c>
-      <c r="D30" t="str">
-        <v>Floating chat bubble rendered</v>
-      </c>
-      <c r="E30" t="str">
-        <v>Floating Eco-Assistant chatbot bubble rendered at bottom-right with pulse animation</v>
-      </c>
-      <c r="F30" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="G30" t="str">
-        <v>13/6/2026, 10:35:28 am</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="str">
-        <v>TC-30</v>
-      </c>
-      <c r="B31" t="str">
-        <v>AI Chatbot</v>
-      </c>
-      <c r="C31" t="str">
-        <v>Chatbot opens and shows welcome message</v>
-      </c>
-      <c r="D31" t="str">
-        <v>Chat pane opens with "Eco-Bot" welcome message</v>
-      </c>
-      <c r="E31" t="str">
-        <v>Chat pane opened with Eco-Bot welcome message, quick prompt chips, and input form</v>
-      </c>
-      <c r="F31" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="G31" t="str">
-        <v>13/6/2026, 10:35:30 am</v>
+        <v>18/6/2026, 1:44:32 pm</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G29"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1183,7 +1137,7 @@
         <v>Test Date</v>
       </c>
       <c r="B6" t="str">
-        <v>13/6/2026</v>
+        <v>18/6/2026</v>
       </c>
     </row>
     <row r="7">
@@ -1191,7 +1145,7 @@
         <v>Start Time</v>
       </c>
       <c r="B7" t="str">
-        <v>10:33:59 am</v>
+        <v>1:39:35 pm</v>
       </c>
     </row>
     <row r="8">
@@ -1199,7 +1153,7 @@
         <v>End Time</v>
       </c>
       <c r="B8" t="str">
-        <v>10:35:30 am</v>
+        <v>1:44:33 pm</v>
       </c>
     </row>
     <row r="9">
@@ -1207,7 +1161,7 @@
         <v>Duration</v>
       </c>
       <c r="B9" t="str">
-        <v>1m 31s</v>
+        <v>4m 57s</v>
       </c>
     </row>
     <row r="10">
@@ -1215,7 +1169,7 @@
         <v>Total Test Cases</v>
       </c>
       <c r="B10">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11">
@@ -1223,7 +1177,7 @@
         <v>Passed</v>
       </c>
       <c r="B11">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -1231,7 +1185,7 @@
         <v>Failed</v>
       </c>
       <c r="B12">
-        <v>0</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13">
@@ -1239,7 +1193,7 @@
         <v>Pass Rate</v>
       </c>
       <c r="B13" t="str">
-        <v>100.0%</v>
+        <v>3.6%</v>
       </c>
     </row>
     <row r="14">
@@ -1298,16 +1252,16 @@
         <v>Authentication</v>
       </c>
       <c r="B2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C2">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E2" t="str">
-        <v>100%</v>
+        <v>25%</v>
       </c>
     </row>
     <row r="3">
@@ -1318,13 +1272,13 @@
         <v>6</v>
       </c>
       <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
         <v>6</v>
       </c>
-      <c r="D3">
-        <v>0</v>
-      </c>
       <c r="E3" t="str">
-        <v>100%</v>
+        <v>0%</v>
       </c>
     </row>
     <row r="4">
@@ -1335,13 +1289,13 @@
         <v>6</v>
       </c>
       <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
         <v>6</v>
       </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
       <c r="E4" t="str">
-        <v>100%</v>
+        <v>0%</v>
       </c>
     </row>
     <row r="5">
@@ -1352,13 +1306,13 @@
         <v>4</v>
       </c>
       <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
         <v>4</v>
       </c>
-      <c r="D5">
-        <v>0</v>
-      </c>
       <c r="E5" t="str">
-        <v>100%</v>
+        <v>0%</v>
       </c>
     </row>
     <row r="6">
@@ -1369,13 +1323,13 @@
         <v>3</v>
       </c>
       <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
         <v>3</v>
       </c>
-      <c r="D6">
-        <v>0</v>
-      </c>
       <c r="E6" t="str">
-        <v>100%</v>
+        <v>0%</v>
       </c>
     </row>
     <row r="7">
@@ -1386,13 +1340,13 @@
         <v>3</v>
       </c>
       <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
         <v>3</v>
       </c>
-      <c r="D7">
-        <v>0</v>
-      </c>
       <c r="E7" t="str">
-        <v>100%</v>
+        <v>0%</v>
       </c>
     </row>
     <row r="8">
@@ -1403,13 +1357,13 @@
         <v>2</v>
       </c>
       <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8">
         <v>2</v>
       </c>
-      <c r="D8">
-        <v>0</v>
-      </c>
       <c r="E8" t="str">
-        <v>100%</v>
+        <v>0%</v>
       </c>
     </row>
   </sheetData>

</xml_diff>